<commit_message>
Various discrete emissions added (restoration interventions, mulching etc)
</commit_message>
<xml_diff>
--- a/Templates/alpha_wp.xlsx
+++ b/Templates/alpha_wp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFCB6B4-CB91-41C8-A072-F1B6ED8F5489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6633BE33-9BCB-4035-8334-BCA657A38A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>Compartment</t>
   </si>
@@ -81,6 +81,12 @@
   </si>
   <si>
     <t>Buried</t>
+  </si>
+  <si>
+    <t>IPCC default half-lives</t>
+  </si>
+  <si>
+    <t>Values from v2.12 sub model</t>
   </si>
 </sst>
 </file>
@@ -398,15 +404,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -419,8 +427,14 @@
       <c r="D1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -431,10 +445,17 @@
         <v>5</v>
       </c>
       <c r="D2">
+        <f>E2/LN(2)</f>
+        <v>2.8853900817779268</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
         <v>0.20895</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -445,10 +466,17 @@
         <v>6</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D4" si="0">E3/LN(2)</f>
+        <v>36.067376022224089</v>
+      </c>
+      <c r="E3">
+        <v>25</v>
+      </c>
+      <c r="F3">
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -459,10 +487,17 @@
         <v>7</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
+        <v>50.49432643111372</v>
+      </c>
+      <c r="E4">
+        <v>35</v>
+      </c>
+      <c r="F4">
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -476,7 +511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -490,7 +525,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Prepping for update to biofuel modelling
</commit_message>
<xml_diff>
--- a/Templates/alpha_wp.xlsx
+++ b/Templates/alpha_wp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://forestresearch-my.sharepoint.com/personal/jacob_osullivan_forestresearch_gov_uk/Documents/Turbines and trees/CCWoP/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6633BE33-9BCB-4035-8334-BCA657A38A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{6633BE33-9BCB-4035-8334-BCA657A38A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{061EF96B-6239-43D1-97FC-FC89590FA7E1}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
   <si>
     <t>Compartment</t>
   </si>
@@ -74,19 +74,22 @@
     <t>Unprocessed</t>
   </si>
   <si>
-    <t>Mulch/foliage</t>
-  </si>
-  <si>
     <t>Stemwood</t>
   </si>
   <si>
-    <t>Buried</t>
-  </si>
-  <si>
-    <t>IPCC default half-lives</t>
-  </si>
-  <si>
-    <t>Values from v2.12 sub model</t>
+    <t>Half-life</t>
+  </si>
+  <si>
+    <t>Foliage</t>
+  </si>
+  <si>
+    <t>Roots</t>
+  </si>
+  <si>
+    <t>Brash</t>
+  </si>
+  <si>
+    <t>alpha_wpB</t>
   </si>
 </sst>
 </file>
@@ -404,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" bestFit="1" customWidth="1"/>
@@ -414,7 +417,7 @@
     <col min="6" max="6" width="25.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -428,13 +431,10 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -445,17 +445,14 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <f>E2/LN(2)</f>
-        <v>2.8853900817779268</v>
+        <f>LN(2)/E2</f>
+        <v>0.34657359027997264</v>
       </c>
       <c r="E2">
         <v>2</v>
       </c>
-      <c r="F2">
-        <v>0.20895</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -466,17 +463,14 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D4" si="0">E3/LN(2)</f>
-        <v>36.067376022224089</v>
+        <f t="shared" ref="D3:D8" si="0">LN(2)/E3</f>
+        <v>2.7725887222397813E-2</v>
       </c>
       <c r="E3">
         <v>25</v>
       </c>
-      <c r="F3">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -488,55 +482,82 @@
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>50.49432643111372</v>
+        <v>1.980420515885558E-2</v>
       </c>
       <c r="E4">
         <v>35</v>
       </c>
-      <c r="F4">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
+        <v>0.34657359027997264</v>
+      </c>
+      <c r="E5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
       </c>
       <c r="D6">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>5.3319013889226559E-2</v>
+      </c>
+      <c r="E6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7">
-        <v>120</v>
+        <f t="shared" si="0"/>
+        <v>3.6481430555786593E-2</v>
+      </c>
+      <c r="E7">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>6.9314718055994526E-2</v>
+      </c>
+      <c r="E8">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Decay of timber/brash left on site added
</commit_message>
<xml_diff>
--- a/Templates/alpha_wp.xlsx
+++ b/Templates/alpha_wp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://forestresearch-my.sharepoint.com/personal/jacob_osullivan_forestresearch_gov_uk/Documents/Turbines and trees/CCWoP/Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{6633BE33-9BCB-4035-8334-BCA657A38A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{061EF96B-6239-43D1-97FC-FC89590FA7E1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C4F3DE-F393-4AF4-9A78-670E248DA34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Compartment</t>
   </si>
@@ -89,7 +89,16 @@
     <t>Brash</t>
   </si>
   <si>
-    <t>alpha_wpB</t>
+    <t>alpha_s</t>
+  </si>
+  <si>
+    <t>alpha_f</t>
+  </si>
+  <si>
+    <t>alpha_r</t>
+  </si>
+  <si>
+    <t>alpha_b</t>
   </si>
 </sst>
 </file>
@@ -496,7 +505,7 @@
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
@@ -514,7 +523,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6">
         <f t="shared" si="0"/>
@@ -532,7 +541,7 @@
         <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
@@ -550,7 +559,7 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D8">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Offcuts and foliage added to wood product decays
</commit_message>
<xml_diff>
--- a/Templates/alpha_wp.xlsx
+++ b/Templates/alpha_wp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C4F3DE-F393-4AF4-9A78-670E248DA34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF338F49-92CB-469D-A54A-2291D8E7F967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>Compartment</t>
   </si>
@@ -86,9 +86,6 @@
     <t>Roots</t>
   </si>
   <si>
-    <t>Brash</t>
-  </si>
-  <si>
     <t>alpha_s</t>
   </si>
   <si>
@@ -99,6 +96,24 @@
   </si>
   <si>
     <t>alpha_b</t>
+  </si>
+  <si>
+    <t>Mulch</t>
+  </si>
+  <si>
+    <t>alpha_m</t>
+  </si>
+  <si>
+    <t>Branches</t>
+  </si>
+  <si>
+    <t>Offcuts</t>
+  </si>
+  <si>
+    <t>alpha_wpO</t>
+  </si>
+  <si>
+    <t>delta</t>
   </si>
 </sst>
 </file>
@@ -416,17 +431,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -442,8 +457,11 @@
       <c r="E1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -460,8 +478,11 @@
       <c r="E2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -472,14 +493,17 @@
         <v>6</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D8" si="0">LN(2)/E3</f>
+        <f t="shared" ref="D3:D10" si="0">LN(2)/E3</f>
         <v>2.7725887222397813E-2</v>
       </c>
       <c r="E3">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -496,77 +520,134 @@
       <c r="E4">
         <v>35</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>0.34657359027997264</v>
+        <v>0.24843984966306282</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>2.79</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>17</v>
       </c>
       <c r="D6">
         <f t="shared" si="0"/>
-        <v>5.3319013889226559E-2</v>
+        <v>0.56353429313816694</v>
       </c>
       <c r="E6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+        <v>1.23</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>3.6481430555786593E-2</v>
+        <v>5.3319013889226559E-2</v>
       </c>
       <c r="E7">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8">
         <f t="shared" si="0"/>
-        <v>6.9314718055994526E-2</v>
+        <v>3.6481430555786593E-2</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>19</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9">
+        <f t="shared" ref="D9" si="1">LN(2)/E9</f>
+        <v>0.24843984966306282</v>
+      </c>
+      <c r="E9">
+        <v>2.79</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>0.24843984966306282</v>
+      </c>
+      <c r="E10">
+        <v>2.79</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>